<commit_message>
Reorder Excel sheet so director is listed first
</commit_message>
<xml_diff>
--- a/movies.xlsx
+++ b/movies.xlsx
@@ -430,9 +430,9 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
@@ -440,17 +440,17 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Director</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -467,17 +467,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Jerzy Hoffman</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>The Deluge</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>1974</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Jerzy Hoffman</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -494,17 +494,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Jerzy Hoffman</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>With Fire and Sword</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>1999</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Jerzy Hoffman</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -521,17 +521,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Aleksander Ford</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Knights of the Teutonic Order</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1960</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Aleksander Ford</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
Update get_director output formatting
</commit_message>
<xml_diff>
--- a/movies.xlsx
+++ b/movies.xlsx
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jerzy Hoffman</t>
+          <t>Hoffman, Jerzy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jerzy Hoffman</t>
+          <t>Hoffman, Jerzy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aleksander Ford</t>
+          <t>Ford, Aleksander</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Update code so that each genre gets its own column and we denote if the movie has said genre via a checkbox
</commit_message>
<xml_diff>
--- a/movies.xlsx
+++ b/movies.xlsx
@@ -1,42 +1,126 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Movies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Movies" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Movies'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Movies!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+  <si>
+    <t>Director</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Genres</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>Adventure</t>
+  </si>
+  <si>
+    <t>War</t>
+  </si>
+  <si>
+    <t>Romance</t>
+  </si>
+  <si>
+    <t>Drama</t>
+  </si>
+  <si>
+    <t>Hoffman, Jerzy</t>
+  </si>
+  <si>
+    <t>The Deluge</t>
+  </si>
+  <si>
+    <t>1974</t>
+  </si>
+  <si>
+    <t>Poland, Soviet Union</t>
+  </si>
+  <si>
+    <t>History, Adventure, War, Romance</t>
+  </si>
+  <si>
+    <t>With Fire and Sword</t>
+  </si>
+  <si>
+    <t>1999</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>War, Romance, Drama</t>
+  </si>
+  <si>
+    <t>Ford, Aleksander</t>
+  </si>
+  <si>
+    <t>Knights of the Teutonic Order</t>
+  </si>
+  <si>
+    <t>1960</t>
+  </si>
+  <si>
+    <t>Adventure, Drama, History, War</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -48,94 +132,66 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -422,131 +478,148 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="30.7109375" customWidth="1"/>
+    <col min="5" max="5" width="40.7109375" customWidth="1"/>
+    <col min="6" max="10" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Director</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Genres</t>
-        </is>
+    <row r="1" spans="1:10" ht="25" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hoffman, Jerzy</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>The Deluge</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1974</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Poland, Soviet Union</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>History, Adventure, War, Romance</t>
-        </is>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hoffman, Jerzy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>With Fire and Sword</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1999</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>War, Romance, Drama</t>
-        </is>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ford, Aleksander</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Knights of the Teutonic Order</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1960</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Adventure, Drama, History, War</t>
-        </is>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:J4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>